<commit_message>
Mark Radyo D as removed in tracking workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QDWreot8xbQDcQ1H1i42Zr
</commit_message>
<xml_diff>
--- a/canliradyodinle-radyo-takip.xlsx
+++ b/canliradyodinle-radyo-takip.xlsx
@@ -4830,14 +4830,14 @@
     </row>
     <row r="388" ht="15" customHeight="1" s="30">
       <c r="A388" s="35" t="n"/>
-      <c r="B388" s="51" t="inlineStr">
+      <c r="B388" s="47" t="inlineStr">
         <is>
           <t>Radyo D</t>
         </is>
       </c>
-      <c r="C388" s="52" t="inlineStr">
-        <is>
-          <t>13.10.2026'da eklendi (logo: resmi sitede büyük logo yok, canliradyodinle.fm logosu kullanıldı)</t>
+      <c r="C388" s="48" t="inlineStr">
+        <is>
+          <t>13.10.2026'da eklendi, aynı gün sitemizden kaldırıldı (silindi).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mark five Adana radios as live in tracking workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016qBi94VY85r4H3aYhrfsx3
</commit_message>
<xml_diff>
--- a/canliradyodinle-radyo-takip.xlsx
+++ b/canliradyodinle-radyo-takip.xlsx
@@ -5392,27 +5392,27 @@
     </row>
     <row r="438" ht="15" customHeight="1" s="30">
       <c r="A438" s="35" t="n"/>
-      <c r="B438" s="38" t="inlineStr">
+      <c r="B438" s="36" t="inlineStr">
         <is>
           <t>Adana FM</t>
         </is>
       </c>
-      <c r="C438" s="39" t="inlineStr">
-        <is>
-          <t>13.10.2026'da eklendi (onay:0, logo yüklendi); yayına alınmayı (onay:1) ve yayın testini bekliyor. Resmi logo.</t>
+      <c r="C438" s="37" t="inlineStr">
+        <is>
+          <t>13.10.2026'da eklendi ve yayına alındı (player 3, yayın testi OK). Resmi logo 500x500.</t>
         </is>
       </c>
     </row>
     <row r="439" ht="15" customHeight="1" s="30">
       <c r="A439" s="35" t="n"/>
-      <c r="B439" s="38" t="inlineStr">
+      <c r="B439" s="36" t="inlineStr">
         <is>
           <t>Adana Kozan Fm</t>
         </is>
       </c>
-      <c r="C439" s="39" t="inlineStr">
-        <is>
-          <t>13.10.2026'da eklendi (onay:0, logo yüklendi); yayına alınmayı (onay:1) ve yayın testini bekliyor. Sitede adı: Kozan FM. Logo canliradyodinle.fm'den.</t>
+      <c r="C439" s="37" t="inlineStr">
+        <is>
+          <t>13.10.2026'da eklendi ve yayına alındı (player 3, yayın testi OK). Sitede adı: Kozan FM. Logo canliradyodinle.fm'den.</t>
         </is>
       </c>
     </row>
@@ -5457,27 +5457,27 @@
     </row>
     <row r="443" ht="15" customHeight="1" s="30">
       <c r="A443" s="35" t="n"/>
-      <c r="B443" s="38" t="inlineStr">
+      <c r="B443" s="36" t="inlineStr">
         <is>
           <t>Adana Radyo Başkent</t>
         </is>
       </c>
-      <c r="C443" s="39" t="inlineStr">
-        <is>
-          <t>13.10.2026'da eklendi (onay:0, logo yüklendi); yayına alınmayı (onay:1) ve yayın testini bekliyor. Sitede adı: Radyo Başkent Adana. Logo canliradyodinle.fm'den.</t>
+      <c r="C443" s="37" t="inlineStr">
+        <is>
+          <t>13.10.2026'da eklendi ve yayına alındı (player 3, yayın testi OK). Sitede adı: Radyo Başkent Adana. Logo canliradyodinle.fm'den.</t>
         </is>
       </c>
     </row>
     <row r="444" ht="15" customHeight="1" s="30">
       <c r="A444" s="35" t="n"/>
-      <c r="B444" s="38" t="inlineStr">
+      <c r="B444" s="36" t="inlineStr">
         <is>
           <t>Adana Radyo Çukurova</t>
         </is>
       </c>
-      <c r="C444" s="39" t="inlineStr">
-        <is>
-          <t>13.10.2026'da eklendi (onay:0, logo yüklendi); yayına alınmayı (onay:1) ve yayın testini bekliyor. Sitede adı: Radyo Çukurova. Resmi logo.</t>
+      <c r="C444" s="37" t="inlineStr">
+        <is>
+          <t>13.10.2026'da eklendi ve yayına alındı (player 3, yayın testi OK). Sitede adı: Radyo Çukurova. Resmi logo 500x500.</t>
         </is>
       </c>
     </row>
@@ -5501,14 +5501,14 @@
     </row>
     <row r="447" ht="15" customHeight="1" s="30">
       <c r="A447" s="35" t="n"/>
-      <c r="B447" s="38" t="inlineStr">
+      <c r="B447" s="36" t="inlineStr">
         <is>
           <t>Akdeniz FM 105.7</t>
         </is>
       </c>
-      <c r="C447" s="39" t="inlineStr">
-        <is>
-          <t>13.10.2026'da eklendi (onay:0, logo yüklendi); yayına alınmayı (onay:1) ve yayın testini bekliyor. Sitede adı: Akdeniz FM Adana. Logo canliradyodinle.fm'den.</t>
+      <c r="C447" s="37" t="inlineStr">
+        <is>
+          <t>13.10.2026'da eklendi ve yayına alındı (player 3, yayın testi OK). Sitede adı: Akdeniz FM Adana. Logo canliradyodinle.fm'den.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Radyo Erkan and Adana Süper FM to tracking workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016qBi94VY85r4H3aYhrfsx3
</commit_message>
<xml_diff>
--- a/canliradyodinle-radyo-takip.xlsx
+++ b/canliradyodinle-radyo-takip.xlsx
@@ -5483,21 +5483,29 @@
     </row>
     <row r="445" ht="15" customHeight="1" s="30">
       <c r="A445" s="35" t="n"/>
-      <c r="B445" s="47" t="inlineStr">
+      <c r="B445" s="36" t="inlineStr">
         <is>
           <t>Adana Radyo Erkan</t>
         </is>
       </c>
-      <c r="C445" s="48" t="n"/>
+      <c r="C445" s="37" t="inlineStr">
+        <is>
+          <t>13.10.2026'da eklendi ve yayına alındı (player 3, yayın testi OK). Sitede adı: Radyo Erkan. Logo canliradyodinle.fm'den.</t>
+        </is>
+      </c>
     </row>
     <row r="446" ht="15" customHeight="1" s="30">
       <c r="A446" s="35" t="n"/>
-      <c r="B446" s="47" t="inlineStr">
+      <c r="B446" s="36" t="inlineStr">
         <is>
           <t>Adana Süper FM</t>
         </is>
       </c>
-      <c r="C446" s="48" t="n"/>
+      <c r="C446" s="37" t="inlineStr">
+        <is>
+          <t>13.10.2026'da eklendi ve yayına alındı (player 3, yayın testi OK). Logo canliradyodinle.fm'den.</t>
+        </is>
+      </c>
     </row>
     <row r="447" ht="15" customHeight="1" s="30">
       <c r="A447" s="35" t="n"/>
@@ -5519,7 +5527,11 @@
           <t>CRT FM</t>
         </is>
       </c>
-      <c r="C448" s="48" t="n"/>
+      <c r="C448" s="48" t="inlineStr">
+        <is>
+          <t>Eklenmedi: yayını sitemizdeki Radyo 01 ile aynı (stream.turkiyeradyolari.com/01fm, yayın adı CRT FM 103.1).</t>
+        </is>
+      </c>
     </row>
     <row r="449" ht="15" customHeight="1" s="30">
       <c r="A449" s="35" t="n"/>

</xml_diff>

<commit_message>
Note redesigned logos for Adana radios in tracking workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016qBi94VY85r4H3aYhrfsx3
</commit_message>
<xml_diff>
--- a/canliradyodinle-radyo-takip.xlsx
+++ b/canliradyodinle-radyo-takip.xlsx
@@ -5399,7 +5399,7 @@
       </c>
       <c r="C438" s="37" t="inlineStr">
         <is>
-          <t>13.10.2026'da eklendi ve yayına alındı (player 3, yayın testi OK). Resmi logo 500x500.</t>
+          <t>13.10.2026'da eklendi ve yayına alındı (player 3, yayın testi OK). Logo tarafımızdan tasarlandı (500x500, beyaz zemin).</t>
         </is>
       </c>
     </row>
@@ -5412,7 +5412,7 @@
       </c>
       <c r="C439" s="37" t="inlineStr">
         <is>
-          <t>13.10.2026'da eklendi ve yayına alındı (player 3, yayın testi OK). Sitede adı: Kozan FM. Logo canliradyodinle.fm'den.</t>
+          <t>13.10.2026'da eklendi ve yayına alındı (player 3, yayın testi OK). Sitede adı: Kozan FM. Logo tarafımızdan tasarlandı (500x500, beyaz zemin).</t>
         </is>
       </c>
     </row>
@@ -5464,7 +5464,7 @@
       </c>
       <c r="C443" s="37" t="inlineStr">
         <is>
-          <t>13.10.2026'da eklendi ve yayına alındı (player 3, yayın testi OK). Sitede adı: Radyo Başkent Adana. Logo canliradyodinle.fm'den.</t>
+          <t>13.10.2026'da eklendi ve yayına alındı (player 3, yayın testi OK). Sitede adı: Radyo Başkent Adana. Logo tarafımızdan tasarlandı (500x500, beyaz zemin).</t>
         </is>
       </c>
     </row>
@@ -5477,7 +5477,7 @@
       </c>
       <c r="C444" s="37" t="inlineStr">
         <is>
-          <t>13.10.2026'da eklendi ve yayına alındı (player 3, yayın testi OK). Sitede adı: Radyo Çukurova. Resmi logo 500x500.</t>
+          <t>13.10.2026'da eklendi ve yayına alındı (player 3, yayın testi OK). Sitede adı: Radyo Çukurova. Resmi logo (büyütülmeden).</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="C445" s="37" t="inlineStr">
         <is>
-          <t>13.10.2026'da eklendi ve yayına alındı (player 3, yayın testi OK). Sitede adı: Radyo Erkan. Logo canliradyodinle.fm'den.</t>
+          <t>13.10.2026'da eklendi ve yayına alındı (player 3, yayın testi OK). Sitede adı: Radyo Erkan. Logo tarafımızdan tasarlandı (500x500, beyaz zemin).</t>
         </is>
       </c>
     </row>
@@ -5503,7 +5503,7 @@
       </c>
       <c r="C446" s="37" t="inlineStr">
         <is>
-          <t>13.10.2026'da eklendi ve yayına alındı (player 3, yayın testi OK). Logo canliradyodinle.fm'den.</t>
+          <t>13.10.2026'da eklendi ve yayına alındı (player 3, yayın testi OK). Logo tarafımızdan tasarlandı (500x500, beyaz zemin).</t>
         </is>
       </c>
     </row>
@@ -5516,7 +5516,7 @@
       </c>
       <c r="C447" s="37" t="inlineStr">
         <is>
-          <t>13.10.2026'da eklendi ve yayına alındı (player 3, yayın testi OK). Sitede adı: Akdeniz FM Adana. Logo canliradyodinle.fm'den.</t>
+          <t>13.10.2026'da eklendi ve yayına alındı (player 3, yayın testi OK). Sitede adı: Akdeniz FM Adana. Logo tarafımızdan tasarlandı (500x500, beyaz zemin).</t>
         </is>
       </c>
     </row>

</xml_diff>